<commit_message>
Align the Weekly Tracker with the schedule (assigned, done, how much)
</commit_message>
<xml_diff>
--- a/mentor-tracking-sheet/Dev Weekend - Mentee Tracker.xlsx
+++ b/mentor-tracking-sheet/Dev Weekend - Mentee Tracker.xlsx
@@ -551,11 +551,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="96" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -604,7 +604,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Weekly Tracker is what you fill each week. Every week has a dated bar with all mentees under it. For each mentee write the tasks you discussed, mark how much they did, and give points out of 10.</t>
+          <t>Weekly Tracker is what you fill each week, in line with the schedule. For each mentee, mark how many of the five weekday days they did each habit and talk, what core work was assigned and how much got done, the weekend grind hours, and give points out of 10.</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Daily Log is day-by-day habits and tasks. 1-on-1 Log is for sessions, with who logged it.</t>
+          <t>Daily Log is the day-by-day version of the same schedule. 1-on-1 Log is for sessions.</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Each new week</t>
+          <t>The schedule it follows</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr"/>
@@ -660,7 +660,7 @@
       <c r="A13" s="3" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Each blue bar is a new week, dated. Under it the same mentees are copied in as ready rows, so you just fill the week. Weeks are laid out ahead, copy the last block to add more.</t>
+          <t>Weekdays run journaling, morning reading, the Mindset talk at breakfast, core work, the Engineering talk at lunch, and the Dean talk at dinner. Weekends are the ten-hour grind plus family time. The weekly columns line up with exactly that.</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Built to import into Pathment later</t>
+          <t>What was assigned, done, and how much</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
@@ -680,7 +680,7 @@
       <c r="A16" s="3" t="inlineStr"/>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Keep the header rows and the dropdown values as they are, one mentee per row, and Pathment will import this sheet straight in when it is ready. Email is the key that links a mentee across tabs. See import-format.md.</t>
+          <t>For the habits and talks, the target is the five weekday days, so 4 out of 5 means four days done. For core work you write what was assigned, what they completed, and the percent done. For the grind, hours out of ten. That is the assigned, completed, and how-much, in line with the schedule.</t>
         </is>
       </c>
     </row>
@@ -691,141 +691,89 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>What the columns mean</t>
+          <t>Built to import into Pathment later</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Tasks discussed</t>
-        </is>
-      </c>
+      <c r="A19" s="3" t="inlineStr"/>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>What you agreed the mentee would do this week.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Tasks done</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>What they actually got through.</t>
+          <t>Keep the headers and dropdown values as they are, one mentee per row. Email is the key that links a mentee across tabs. See import-format.md.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Done %</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>How much of the discussed tasks they completed, 0 to 100.</t>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>At a glance (updates from the tracker)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Points (/10)</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Your mark for the week against what was discussed. Effort and outcome together.</t>
-        </is>
+          <t>Mentees tracked</t>
+        </is>
+      </c>
+      <c r="B22" s="6">
+        <f>COUNTA('Mentee Tracker'!A2:A200)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>On track, Watch, or At risk. Colour-coded so the people who need you stand out.</t>
-        </is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
+        <f>COUNTIF('Mentee Tracker'!N2:N200,"On track")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="B24" s="6">
+        <f>COUNTIF('Mentee Tracker'!N2:N200,"Watch")</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>At a glance (updates from the tracker)</t>
-        </is>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="B25" s="6">
+        <f>COUNTIF('Mentee Tracker'!N2:N200,"At risk")</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Mentees tracked</t>
+          <t>Average on-time %</t>
         </is>
       </c>
       <c r="B26" s="6">
-        <f>COUNTA('Mentee Tracker'!A2:A200)</f>
+        <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!K2:K200),0),0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>On track</t>
+          <t>Average points (filled weeks)</t>
         </is>
       </c>
       <c r="B27" s="6">
-        <f>COUNTIF('Mentee Tracker'!N2:N200,"On track")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Watch</t>
-        </is>
-      </c>
-      <c r="B28" s="6">
-        <f>COUNTIF('Mentee Tracker'!N2:N200,"Watch")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>At risk</t>
-        </is>
-      </c>
-      <c r="B29" s="6">
-        <f>COUNTIF('Mentee Tracker'!N2:N200,"At risk")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>Average on-time %</t>
-        </is>
-      </c>
-      <c r="B30" s="6">
-        <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!K2:K200),0),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>Average points (latest week)</t>
-        </is>
-      </c>
-      <c r="B31" s="6">
-        <f>IFERROR(ROUND(AVERAGEIF('Weekly Tracker'!H2:H1000,"&gt;0"),1),0)</f>
+        <f>IFERROR(ROUND(AVERAGEIF('Weekly Tracker'!N2:N2000,"&gt;0"),1),0)</f>
         <v/>
       </c>
     </row>
@@ -840,22 +788,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:P85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Week of</t>
@@ -873,35 +827,65 @@
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Journaling /5</t>
         </is>
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>Tasks discussed</t>
+          <t>Reading /5</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>Tasks done</t>
+          <t>Mindset talk /5</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">
         <is>
-          <t>Done %</t>
+          <t>Eng. talk /5</t>
         </is>
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
-          <t>Points (/10)</t>
+          <t>Dean talk /5</t>
         </is>
       </c>
       <c r="I1" s="7" t="inlineStr">
         <is>
+          <t>Core work assigned</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Core work completed</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Core %</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Grind h /10</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Family time</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>Points /10</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>Feedback / focus for next week</t>
         </is>
@@ -928,33 +912,51 @@
           <t>aisha.k@email.com</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>Add authentication (JWT)</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>Auth started, refresh-token flow next</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>Finish CRUD API, start auth (JWT)</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>CRUD API done, auth started</t>
-        </is>
-      </c>
-      <c r="G3" s="11" t="n">
-        <v>80</v>
-      </c>
-      <c r="H3" s="11" t="n">
+      <c r="N3" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="O3" s="11" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="J3" s="12" t="inlineStr">
+      <c r="P3" s="12" t="inlineStr">
         <is>
           <t>Strong week. Pair on auth Thursday.</t>
         </is>
@@ -974,33 +976,51 @@
           <t>diego.m@email.com</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>Component composition</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>Reading done, dashboard in late</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Component composition, responsive dashboard</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>Dashboard in (late), composition reading done</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>60</v>
-      </c>
-      <c r="H4" s="11" t="n">
+      <c r="N4" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="O4" s="11" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="P4" s="12" t="inlineStr">
         <is>
           <t>Good effort against real constraints. Protect deadlines.</t>
         </is>
@@ -1020,35 +1040,53 @@
           <t>priya.n@email.com</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Excused</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>API integration, REST best-practices reading</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="D5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>API integration exercise</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>Little progress, re-engaging</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="K5" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="L5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="O5" s="11" t="inlineStr">
         <is>
           <t>At risk</t>
         </is>
       </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>Warm check-in done. Small wins first, light load next week.</t>
+      <c r="P5" s="12" t="inlineStr">
+        <is>
+          <t>Warm check-in done. Lighter load next week, small wins first.</t>
         </is>
       </c>
     </row>
@@ -1066,35 +1104,53 @@
           <t>liam.w@email.com</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>Auth middleware + rate-limit stretch</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Middleware done early</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Auth middleware, rate-limiting stretch</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>Auth middleware done early</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="11" t="n">
+      <c r="N6" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="O6" s="11" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr">
-        <is>
-          <t>Way ahead. Add a real stretch so he is challenged.</t>
+      <c r="P6" s="12" t="inlineStr">
+        <is>
+          <t>Way ahead. Give him a real stretch.</t>
         </is>
       </c>
     </row>
@@ -1112,35 +1168,53 @@
           <t>fatima.n@email.com</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>Async/await refactor</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>In progress, event-loop reading done</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Async/await refactor, event loop reading</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>Refactor in progress, reading done</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>75</v>
-      </c>
-      <c r="H7" s="11" t="n">
+      <c r="N7" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="O7" s="11" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>Climbing nicely. Unblock async/await and keep going.</t>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>Climbing nicely. Unblock async/await.</t>
         </is>
       </c>
     </row>
@@ -1158,33 +1232,51 @@
           <t>tomas.b@email.com</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Form validation library</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Submitted late, regex quiz pending</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Validation library, regex quiz</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>Library in (late), quiz pending</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>55</v>
-      </c>
-      <c r="H8" s="11" t="n">
+      <c r="N8" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="O8" s="11" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="J8" s="12" t="inlineStr">
+      <c r="P8" s="12" t="inlineStr">
         <is>
           <t>Slipping a little. Short check-in this week.</t>
         </is>
@@ -1212,12 +1304,18 @@
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr"/>
-      <c r="E10" s="12" t="inlineStr"/>
-      <c r="F10" s="12" t="inlineStr"/>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
       <c r="G10" s="11" t="inlineStr"/>
       <c r="H10" s="11" t="inlineStr"/>
-      <c r="I10" s="11" t="inlineStr"/>
+      <c r="I10" s="12" t="inlineStr"/>
       <c r="J10" s="12" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
+      <c r="L10" s="11" t="inlineStr"/>
+      <c r="M10" s="11" t="inlineStr"/>
+      <c r="N10" s="11" t="inlineStr"/>
+      <c r="O10" s="11" t="inlineStr"/>
+      <c r="P10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -1234,12 +1332,18 @@
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr"/>
-      <c r="E11" s="12" t="inlineStr"/>
-      <c r="F11" s="12" t="inlineStr"/>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
       <c r="G11" s="11" t="inlineStr"/>
       <c r="H11" s="11" t="inlineStr"/>
-      <c r="I11" s="11" t="inlineStr"/>
+      <c r="I11" s="12" t="inlineStr"/>
       <c r="J11" s="12" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr"/>
+      <c r="L11" s="11" t="inlineStr"/>
+      <c r="M11" s="11" t="inlineStr"/>
+      <c r="N11" s="11" t="inlineStr"/>
+      <c r="O11" s="11" t="inlineStr"/>
+      <c r="P11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
@@ -1256,12 +1360,18 @@
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr"/>
-      <c r="E12" s="12" t="inlineStr"/>
-      <c r="F12" s="12" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr"/>
       <c r="H12" s="11" t="inlineStr"/>
-      <c r="I12" s="11" t="inlineStr"/>
+      <c r="I12" s="12" t="inlineStr"/>
       <c r="J12" s="12" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
+      <c r="L12" s="11" t="inlineStr"/>
+      <c r="M12" s="11" t="inlineStr"/>
+      <c r="N12" s="11" t="inlineStr"/>
+      <c r="O12" s="11" t="inlineStr"/>
+      <c r="P12" s="12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
@@ -1278,12 +1388,18 @@
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr"/>
-      <c r="E13" s="12" t="inlineStr"/>
-      <c r="F13" s="12" t="inlineStr"/>
+      <c r="E13" s="11" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr"/>
       <c r="G13" s="11" t="inlineStr"/>
       <c r="H13" s="11" t="inlineStr"/>
-      <c r="I13" s="11" t="inlineStr"/>
+      <c r="I13" s="12" t="inlineStr"/>
       <c r="J13" s="12" t="inlineStr"/>
+      <c r="K13" s="11" t="inlineStr"/>
+      <c r="L13" s="11" t="inlineStr"/>
+      <c r="M13" s="11" t="inlineStr"/>
+      <c r="N13" s="11" t="inlineStr"/>
+      <c r="O13" s="11" t="inlineStr"/>
+      <c r="P13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
@@ -1300,12 +1416,18 @@
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr"/>
-      <c r="E14" s="12" t="inlineStr"/>
-      <c r="F14" s="12" t="inlineStr"/>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
       <c r="G14" s="11" t="inlineStr"/>
       <c r="H14" s="11" t="inlineStr"/>
-      <c r="I14" s="11" t="inlineStr"/>
+      <c r="I14" s="12" t="inlineStr"/>
       <c r="J14" s="12" t="inlineStr"/>
+      <c r="K14" s="11" t="inlineStr"/>
+      <c r="L14" s="11" t="inlineStr"/>
+      <c r="M14" s="11" t="inlineStr"/>
+      <c r="N14" s="11" t="inlineStr"/>
+      <c r="O14" s="11" t="inlineStr"/>
+      <c r="P14" s="12" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
@@ -1322,12 +1444,18 @@
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr"/>
-      <c r="E15" s="12" t="inlineStr"/>
-      <c r="F15" s="12" t="inlineStr"/>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
       <c r="G15" s="11" t="inlineStr"/>
       <c r="H15" s="11" t="inlineStr"/>
-      <c r="I15" s="11" t="inlineStr"/>
+      <c r="I15" s="12" t="inlineStr"/>
       <c r="J15" s="12" t="inlineStr"/>
+      <c r="K15" s="11" t="inlineStr"/>
+      <c r="L15" s="11" t="inlineStr"/>
+      <c r="M15" s="11" t="inlineStr"/>
+      <c r="N15" s="11" t="inlineStr"/>
+      <c r="O15" s="11" t="inlineStr"/>
+      <c r="P15" s="12" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -1351,12 +1479,18 @@
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr"/>
-      <c r="E17" s="12" t="inlineStr"/>
-      <c r="F17" s="12" t="inlineStr"/>
+      <c r="E17" s="11" t="inlineStr"/>
+      <c r="F17" s="11" t="inlineStr"/>
       <c r="G17" s="11" t="inlineStr"/>
       <c r="H17" s="11" t="inlineStr"/>
-      <c r="I17" s="11" t="inlineStr"/>
+      <c r="I17" s="12" t="inlineStr"/>
       <c r="J17" s="12" t="inlineStr"/>
+      <c r="K17" s="11" t="inlineStr"/>
+      <c r="L17" s="11" t="inlineStr"/>
+      <c r="M17" s="11" t="inlineStr"/>
+      <c r="N17" s="11" t="inlineStr"/>
+      <c r="O17" s="11" t="inlineStr"/>
+      <c r="P17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
@@ -1373,12 +1507,18 @@
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr"/>
-      <c r="E18" s="12" t="inlineStr"/>
-      <c r="F18" s="12" t="inlineStr"/>
+      <c r="E18" s="11" t="inlineStr"/>
+      <c r="F18" s="11" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr"/>
       <c r="H18" s="11" t="inlineStr"/>
-      <c r="I18" s="11" t="inlineStr"/>
+      <c r="I18" s="12" t="inlineStr"/>
       <c r="J18" s="12" t="inlineStr"/>
+      <c r="K18" s="11" t="inlineStr"/>
+      <c r="L18" s="11" t="inlineStr"/>
+      <c r="M18" s="11" t="inlineStr"/>
+      <c r="N18" s="11" t="inlineStr"/>
+      <c r="O18" s="11" t="inlineStr"/>
+      <c r="P18" s="12" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
@@ -1395,12 +1535,18 @@
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr"/>
-      <c r="E19" s="12" t="inlineStr"/>
-      <c r="F19" s="12" t="inlineStr"/>
+      <c r="E19" s="11" t="inlineStr"/>
+      <c r="F19" s="11" t="inlineStr"/>
       <c r="G19" s="11" t="inlineStr"/>
       <c r="H19" s="11" t="inlineStr"/>
-      <c r="I19" s="11" t="inlineStr"/>
+      <c r="I19" s="12" t="inlineStr"/>
       <c r="J19" s="12" t="inlineStr"/>
+      <c r="K19" s="11" t="inlineStr"/>
+      <c r="L19" s="11" t="inlineStr"/>
+      <c r="M19" s="11" t="inlineStr"/>
+      <c r="N19" s="11" t="inlineStr"/>
+      <c r="O19" s="11" t="inlineStr"/>
+      <c r="P19" s="12" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
@@ -1417,12 +1563,18 @@
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr"/>
-      <c r="E20" s="12" t="inlineStr"/>
-      <c r="F20" s="12" t="inlineStr"/>
+      <c r="E20" s="11" t="inlineStr"/>
+      <c r="F20" s="11" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr"/>
       <c r="H20" s="11" t="inlineStr"/>
-      <c r="I20" s="11" t="inlineStr"/>
+      <c r="I20" s="12" t="inlineStr"/>
       <c r="J20" s="12" t="inlineStr"/>
+      <c r="K20" s="11" t="inlineStr"/>
+      <c r="L20" s="11" t="inlineStr"/>
+      <c r="M20" s="11" t="inlineStr"/>
+      <c r="N20" s="11" t="inlineStr"/>
+      <c r="O20" s="11" t="inlineStr"/>
+      <c r="P20" s="12" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -1439,12 +1591,18 @@
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr"/>
-      <c r="E21" s="12" t="inlineStr"/>
-      <c r="F21" s="12" t="inlineStr"/>
+      <c r="E21" s="11" t="inlineStr"/>
+      <c r="F21" s="11" t="inlineStr"/>
       <c r="G21" s="11" t="inlineStr"/>
       <c r="H21" s="11" t="inlineStr"/>
-      <c r="I21" s="11" t="inlineStr"/>
+      <c r="I21" s="12" t="inlineStr"/>
       <c r="J21" s="12" t="inlineStr"/>
+      <c r="K21" s="11" t="inlineStr"/>
+      <c r="L21" s="11" t="inlineStr"/>
+      <c r="M21" s="11" t="inlineStr"/>
+      <c r="N21" s="11" t="inlineStr"/>
+      <c r="O21" s="11" t="inlineStr"/>
+      <c r="P21" s="12" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
@@ -1461,12 +1619,18 @@
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr"/>
-      <c r="E22" s="12" t="inlineStr"/>
-      <c r="F22" s="12" t="inlineStr"/>
+      <c r="E22" s="11" t="inlineStr"/>
+      <c r="F22" s="11" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr"/>
       <c r="H22" s="11" t="inlineStr"/>
-      <c r="I22" s="11" t="inlineStr"/>
+      <c r="I22" s="12" t="inlineStr"/>
       <c r="J22" s="12" t="inlineStr"/>
+      <c r="K22" s="11" t="inlineStr"/>
+      <c r="L22" s="11" t="inlineStr"/>
+      <c r="M22" s="11" t="inlineStr"/>
+      <c r="N22" s="11" t="inlineStr"/>
+      <c r="O22" s="11" t="inlineStr"/>
+      <c r="P22" s="12" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
@@ -1490,12 +1654,18 @@
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr"/>
-      <c r="E24" s="12" t="inlineStr"/>
-      <c r="F24" s="12" t="inlineStr"/>
+      <c r="E24" s="11" t="inlineStr"/>
+      <c r="F24" s="11" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr"/>
       <c r="H24" s="11" t="inlineStr"/>
-      <c r="I24" s="11" t="inlineStr"/>
+      <c r="I24" s="12" t="inlineStr"/>
       <c r="J24" s="12" t="inlineStr"/>
+      <c r="K24" s="11" t="inlineStr"/>
+      <c r="L24" s="11" t="inlineStr"/>
+      <c r="M24" s="11" t="inlineStr"/>
+      <c r="N24" s="11" t="inlineStr"/>
+      <c r="O24" s="11" t="inlineStr"/>
+      <c r="P24" s="12" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
@@ -1512,12 +1682,18 @@
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr"/>
-      <c r="E25" s="12" t="inlineStr"/>
-      <c r="F25" s="12" t="inlineStr"/>
+      <c r="E25" s="11" t="inlineStr"/>
+      <c r="F25" s="11" t="inlineStr"/>
       <c r="G25" s="11" t="inlineStr"/>
       <c r="H25" s="11" t="inlineStr"/>
-      <c r="I25" s="11" t="inlineStr"/>
+      <c r="I25" s="12" t="inlineStr"/>
       <c r="J25" s="12" t="inlineStr"/>
+      <c r="K25" s="11" t="inlineStr"/>
+      <c r="L25" s="11" t="inlineStr"/>
+      <c r="M25" s="11" t="inlineStr"/>
+      <c r="N25" s="11" t="inlineStr"/>
+      <c r="O25" s="11" t="inlineStr"/>
+      <c r="P25" s="12" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
@@ -1534,12 +1710,18 @@
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr"/>
-      <c r="E26" s="12" t="inlineStr"/>
-      <c r="F26" s="12" t="inlineStr"/>
+      <c r="E26" s="11" t="inlineStr"/>
+      <c r="F26" s="11" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr"/>
       <c r="H26" s="11" t="inlineStr"/>
-      <c r="I26" s="11" t="inlineStr"/>
+      <c r="I26" s="12" t="inlineStr"/>
       <c r="J26" s="12" t="inlineStr"/>
+      <c r="K26" s="11" t="inlineStr"/>
+      <c r="L26" s="11" t="inlineStr"/>
+      <c r="M26" s="11" t="inlineStr"/>
+      <c r="N26" s="11" t="inlineStr"/>
+      <c r="O26" s="11" t="inlineStr"/>
+      <c r="P26" s="12" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
@@ -1556,12 +1738,18 @@
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr"/>
-      <c r="E27" s="12" t="inlineStr"/>
-      <c r="F27" s="12" t="inlineStr"/>
+      <c r="E27" s="11" t="inlineStr"/>
+      <c r="F27" s="11" t="inlineStr"/>
       <c r="G27" s="11" t="inlineStr"/>
       <c r="H27" s="11" t="inlineStr"/>
-      <c r="I27" s="11" t="inlineStr"/>
+      <c r="I27" s="12" t="inlineStr"/>
       <c r="J27" s="12" t="inlineStr"/>
+      <c r="K27" s="11" t="inlineStr"/>
+      <c r="L27" s="11" t="inlineStr"/>
+      <c r="M27" s="11" t="inlineStr"/>
+      <c r="N27" s="11" t="inlineStr"/>
+      <c r="O27" s="11" t="inlineStr"/>
+      <c r="P27" s="12" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
@@ -1578,12 +1766,18 @@
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr"/>
-      <c r="E28" s="12" t="inlineStr"/>
-      <c r="F28" s="12" t="inlineStr"/>
+      <c r="E28" s="11" t="inlineStr"/>
+      <c r="F28" s="11" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr"/>
       <c r="H28" s="11" t="inlineStr"/>
-      <c r="I28" s="11" t="inlineStr"/>
+      <c r="I28" s="12" t="inlineStr"/>
       <c r="J28" s="12" t="inlineStr"/>
+      <c r="K28" s="11" t="inlineStr"/>
+      <c r="L28" s="11" t="inlineStr"/>
+      <c r="M28" s="11" t="inlineStr"/>
+      <c r="N28" s="11" t="inlineStr"/>
+      <c r="O28" s="11" t="inlineStr"/>
+      <c r="P28" s="12" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
@@ -1600,12 +1794,18 @@
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr"/>
-      <c r="E29" s="12" t="inlineStr"/>
-      <c r="F29" s="12" t="inlineStr"/>
+      <c r="E29" s="11" t="inlineStr"/>
+      <c r="F29" s="11" t="inlineStr"/>
       <c r="G29" s="11" t="inlineStr"/>
       <c r="H29" s="11" t="inlineStr"/>
-      <c r="I29" s="11" t="inlineStr"/>
+      <c r="I29" s="12" t="inlineStr"/>
       <c r="J29" s="12" t="inlineStr"/>
+      <c r="K29" s="11" t="inlineStr"/>
+      <c r="L29" s="11" t="inlineStr"/>
+      <c r="M29" s="11" t="inlineStr"/>
+      <c r="N29" s="11" t="inlineStr"/>
+      <c r="O29" s="11" t="inlineStr"/>
+      <c r="P29" s="12" t="inlineStr"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
@@ -1629,12 +1829,18 @@
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr"/>
-      <c r="E31" s="12" t="inlineStr"/>
-      <c r="F31" s="12" t="inlineStr"/>
+      <c r="E31" s="11" t="inlineStr"/>
+      <c r="F31" s="11" t="inlineStr"/>
       <c r="G31" s="11" t="inlineStr"/>
       <c r="H31" s="11" t="inlineStr"/>
-      <c r="I31" s="11" t="inlineStr"/>
+      <c r="I31" s="12" t="inlineStr"/>
       <c r="J31" s="12" t="inlineStr"/>
+      <c r="K31" s="11" t="inlineStr"/>
+      <c r="L31" s="11" t="inlineStr"/>
+      <c r="M31" s="11" t="inlineStr"/>
+      <c r="N31" s="11" t="inlineStr"/>
+      <c r="O31" s="11" t="inlineStr"/>
+      <c r="P31" s="12" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
@@ -1651,12 +1857,18 @@
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr"/>
-      <c r="E32" s="12" t="inlineStr"/>
-      <c r="F32" s="12" t="inlineStr"/>
+      <c r="E32" s="11" t="inlineStr"/>
+      <c r="F32" s="11" t="inlineStr"/>
       <c r="G32" s="11" t="inlineStr"/>
       <c r="H32" s="11" t="inlineStr"/>
-      <c r="I32" s="11" t="inlineStr"/>
+      <c r="I32" s="12" t="inlineStr"/>
       <c r="J32" s="12" t="inlineStr"/>
+      <c r="K32" s="11" t="inlineStr"/>
+      <c r="L32" s="11" t="inlineStr"/>
+      <c r="M32" s="11" t="inlineStr"/>
+      <c r="N32" s="11" t="inlineStr"/>
+      <c r="O32" s="11" t="inlineStr"/>
+      <c r="P32" s="12" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
@@ -1673,12 +1885,18 @@
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr"/>
-      <c r="E33" s="12" t="inlineStr"/>
-      <c r="F33" s="12" t="inlineStr"/>
+      <c r="E33" s="11" t="inlineStr"/>
+      <c r="F33" s="11" t="inlineStr"/>
       <c r="G33" s="11" t="inlineStr"/>
       <c r="H33" s="11" t="inlineStr"/>
-      <c r="I33" s="11" t="inlineStr"/>
+      <c r="I33" s="12" t="inlineStr"/>
       <c r="J33" s="12" t="inlineStr"/>
+      <c r="K33" s="11" t="inlineStr"/>
+      <c r="L33" s="11" t="inlineStr"/>
+      <c r="M33" s="11" t="inlineStr"/>
+      <c r="N33" s="11" t="inlineStr"/>
+      <c r="O33" s="11" t="inlineStr"/>
+      <c r="P33" s="12" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n">
@@ -1695,12 +1913,18 @@
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr"/>
-      <c r="E34" s="12" t="inlineStr"/>
-      <c r="F34" s="12" t="inlineStr"/>
+      <c r="E34" s="11" t="inlineStr"/>
+      <c r="F34" s="11" t="inlineStr"/>
       <c r="G34" s="11" t="inlineStr"/>
       <c r="H34" s="11" t="inlineStr"/>
-      <c r="I34" s="11" t="inlineStr"/>
+      <c r="I34" s="12" t="inlineStr"/>
       <c r="J34" s="12" t="inlineStr"/>
+      <c r="K34" s="11" t="inlineStr"/>
+      <c r="L34" s="11" t="inlineStr"/>
+      <c r="M34" s="11" t="inlineStr"/>
+      <c r="N34" s="11" t="inlineStr"/>
+      <c r="O34" s="11" t="inlineStr"/>
+      <c r="P34" s="12" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
@@ -1717,12 +1941,18 @@
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr"/>
-      <c r="E35" s="12" t="inlineStr"/>
-      <c r="F35" s="12" t="inlineStr"/>
+      <c r="E35" s="11" t="inlineStr"/>
+      <c r="F35" s="11" t="inlineStr"/>
       <c r="G35" s="11" t="inlineStr"/>
       <c r="H35" s="11" t="inlineStr"/>
-      <c r="I35" s="11" t="inlineStr"/>
+      <c r="I35" s="12" t="inlineStr"/>
       <c r="J35" s="12" t="inlineStr"/>
+      <c r="K35" s="11" t="inlineStr"/>
+      <c r="L35" s="11" t="inlineStr"/>
+      <c r="M35" s="11" t="inlineStr"/>
+      <c r="N35" s="11" t="inlineStr"/>
+      <c r="O35" s="11" t="inlineStr"/>
+      <c r="P35" s="12" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n">
@@ -1739,12 +1969,18 @@
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr"/>
-      <c r="E36" s="12" t="inlineStr"/>
-      <c r="F36" s="12" t="inlineStr"/>
+      <c r="E36" s="11" t="inlineStr"/>
+      <c r="F36" s="11" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr"/>
       <c r="H36" s="11" t="inlineStr"/>
-      <c r="I36" s="11" t="inlineStr"/>
+      <c r="I36" s="12" t="inlineStr"/>
       <c r="J36" s="12" t="inlineStr"/>
+      <c r="K36" s="11" t="inlineStr"/>
+      <c r="L36" s="11" t="inlineStr"/>
+      <c r="M36" s="11" t="inlineStr"/>
+      <c r="N36" s="11" t="inlineStr"/>
+      <c r="O36" s="11" t="inlineStr"/>
+      <c r="P36" s="12" t="inlineStr"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
@@ -1768,12 +2004,18 @@
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr"/>
-      <c r="E38" s="12" t="inlineStr"/>
-      <c r="F38" s="12" t="inlineStr"/>
+      <c r="E38" s="11" t="inlineStr"/>
+      <c r="F38" s="11" t="inlineStr"/>
       <c r="G38" s="11" t="inlineStr"/>
       <c r="H38" s="11" t="inlineStr"/>
-      <c r="I38" s="11" t="inlineStr"/>
+      <c r="I38" s="12" t="inlineStr"/>
       <c r="J38" s="12" t="inlineStr"/>
+      <c r="K38" s="11" t="inlineStr"/>
+      <c r="L38" s="11" t="inlineStr"/>
+      <c r="M38" s="11" t="inlineStr"/>
+      <c r="N38" s="11" t="inlineStr"/>
+      <c r="O38" s="11" t="inlineStr"/>
+      <c r="P38" s="12" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
@@ -1790,12 +2032,18 @@
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr"/>
-      <c r="E39" s="12" t="inlineStr"/>
-      <c r="F39" s="12" t="inlineStr"/>
+      <c r="E39" s="11" t="inlineStr"/>
+      <c r="F39" s="11" t="inlineStr"/>
       <c r="G39" s="11" t="inlineStr"/>
       <c r="H39" s="11" t="inlineStr"/>
-      <c r="I39" s="11" t="inlineStr"/>
+      <c r="I39" s="12" t="inlineStr"/>
       <c r="J39" s="12" t="inlineStr"/>
+      <c r="K39" s="11" t="inlineStr"/>
+      <c r="L39" s="11" t="inlineStr"/>
+      <c r="M39" s="11" t="inlineStr"/>
+      <c r="N39" s="11" t="inlineStr"/>
+      <c r="O39" s="11" t="inlineStr"/>
+      <c r="P39" s="12" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n">
@@ -1812,12 +2060,18 @@
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr"/>
-      <c r="E40" s="12" t="inlineStr"/>
-      <c r="F40" s="12" t="inlineStr"/>
+      <c r="E40" s="11" t="inlineStr"/>
+      <c r="F40" s="11" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr"/>
       <c r="H40" s="11" t="inlineStr"/>
-      <c r="I40" s="11" t="inlineStr"/>
+      <c r="I40" s="12" t="inlineStr"/>
       <c r="J40" s="12" t="inlineStr"/>
+      <c r="K40" s="11" t="inlineStr"/>
+      <c r="L40" s="11" t="inlineStr"/>
+      <c r="M40" s="11" t="inlineStr"/>
+      <c r="N40" s="11" t="inlineStr"/>
+      <c r="O40" s="11" t="inlineStr"/>
+      <c r="P40" s="12" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
@@ -1834,12 +2088,18 @@
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr"/>
-      <c r="E41" s="12" t="inlineStr"/>
-      <c r="F41" s="12" t="inlineStr"/>
+      <c r="E41" s="11" t="inlineStr"/>
+      <c r="F41" s="11" t="inlineStr"/>
       <c r="G41" s="11" t="inlineStr"/>
       <c r="H41" s="11" t="inlineStr"/>
-      <c r="I41" s="11" t="inlineStr"/>
+      <c r="I41" s="12" t="inlineStr"/>
       <c r="J41" s="12" t="inlineStr"/>
+      <c r="K41" s="11" t="inlineStr"/>
+      <c r="L41" s="11" t="inlineStr"/>
+      <c r="M41" s="11" t="inlineStr"/>
+      <c r="N41" s="11" t="inlineStr"/>
+      <c r="O41" s="11" t="inlineStr"/>
+      <c r="P41" s="12" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n">
@@ -1856,12 +2116,18 @@
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr"/>
-      <c r="E42" s="12" t="inlineStr"/>
-      <c r="F42" s="12" t="inlineStr"/>
+      <c r="E42" s="11" t="inlineStr"/>
+      <c r="F42" s="11" t="inlineStr"/>
       <c r="G42" s="11" t="inlineStr"/>
       <c r="H42" s="11" t="inlineStr"/>
-      <c r="I42" s="11" t="inlineStr"/>
+      <c r="I42" s="12" t="inlineStr"/>
       <c r="J42" s="12" t="inlineStr"/>
+      <c r="K42" s="11" t="inlineStr"/>
+      <c r="L42" s="11" t="inlineStr"/>
+      <c r="M42" s="11" t="inlineStr"/>
+      <c r="N42" s="11" t="inlineStr"/>
+      <c r="O42" s="11" t="inlineStr"/>
+      <c r="P42" s="12" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
@@ -1878,12 +2144,18 @@
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr"/>
-      <c r="E43" s="12" t="inlineStr"/>
-      <c r="F43" s="12" t="inlineStr"/>
+      <c r="E43" s="11" t="inlineStr"/>
+      <c r="F43" s="11" t="inlineStr"/>
       <c r="G43" s="11" t="inlineStr"/>
       <c r="H43" s="11" t="inlineStr"/>
-      <c r="I43" s="11" t="inlineStr"/>
+      <c r="I43" s="12" t="inlineStr"/>
       <c r="J43" s="12" t="inlineStr"/>
+      <c r="K43" s="11" t="inlineStr"/>
+      <c r="L43" s="11" t="inlineStr"/>
+      <c r="M43" s="11" t="inlineStr"/>
+      <c r="N43" s="11" t="inlineStr"/>
+      <c r="O43" s="11" t="inlineStr"/>
+      <c r="P43" s="12" t="inlineStr"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
@@ -1907,12 +2179,18 @@
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
-      <c r="E45" s="12" t="inlineStr"/>
-      <c r="F45" s="12" t="inlineStr"/>
+      <c r="E45" s="11" t="inlineStr"/>
+      <c r="F45" s="11" t="inlineStr"/>
       <c r="G45" s="11" t="inlineStr"/>
       <c r="H45" s="11" t="inlineStr"/>
-      <c r="I45" s="11" t="inlineStr"/>
+      <c r="I45" s="12" t="inlineStr"/>
       <c r="J45" s="12" t="inlineStr"/>
+      <c r="K45" s="11" t="inlineStr"/>
+      <c r="L45" s="11" t="inlineStr"/>
+      <c r="M45" s="11" t="inlineStr"/>
+      <c r="N45" s="11" t="inlineStr"/>
+      <c r="O45" s="11" t="inlineStr"/>
+      <c r="P45" s="12" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="n">
@@ -1929,12 +2207,18 @@
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
-      <c r="E46" s="12" t="inlineStr"/>
-      <c r="F46" s="12" t="inlineStr"/>
+      <c r="E46" s="11" t="inlineStr"/>
+      <c r="F46" s="11" t="inlineStr"/>
       <c r="G46" s="11" t="inlineStr"/>
       <c r="H46" s="11" t="inlineStr"/>
-      <c r="I46" s="11" t="inlineStr"/>
+      <c r="I46" s="12" t="inlineStr"/>
       <c r="J46" s="12" t="inlineStr"/>
+      <c r="K46" s="11" t="inlineStr"/>
+      <c r="L46" s="11" t="inlineStr"/>
+      <c r="M46" s="11" t="inlineStr"/>
+      <c r="N46" s="11" t="inlineStr"/>
+      <c r="O46" s="11" t="inlineStr"/>
+      <c r="P46" s="12" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
@@ -1951,12 +2235,18 @@
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
-      <c r="E47" s="12" t="inlineStr"/>
-      <c r="F47" s="12" t="inlineStr"/>
+      <c r="E47" s="11" t="inlineStr"/>
+      <c r="F47" s="11" t="inlineStr"/>
       <c r="G47" s="11" t="inlineStr"/>
       <c r="H47" s="11" t="inlineStr"/>
-      <c r="I47" s="11" t="inlineStr"/>
+      <c r="I47" s="12" t="inlineStr"/>
       <c r="J47" s="12" t="inlineStr"/>
+      <c r="K47" s="11" t="inlineStr"/>
+      <c r="L47" s="11" t="inlineStr"/>
+      <c r="M47" s="11" t="inlineStr"/>
+      <c r="N47" s="11" t="inlineStr"/>
+      <c r="O47" s="11" t="inlineStr"/>
+      <c r="P47" s="12" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n">
@@ -1973,12 +2263,18 @@
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr"/>
-      <c r="E48" s="12" t="inlineStr"/>
-      <c r="F48" s="12" t="inlineStr"/>
+      <c r="E48" s="11" t="inlineStr"/>
+      <c r="F48" s="11" t="inlineStr"/>
       <c r="G48" s="11" t="inlineStr"/>
       <c r="H48" s="11" t="inlineStr"/>
-      <c r="I48" s="11" t="inlineStr"/>
+      <c r="I48" s="12" t="inlineStr"/>
       <c r="J48" s="12" t="inlineStr"/>
+      <c r="K48" s="11" t="inlineStr"/>
+      <c r="L48" s="11" t="inlineStr"/>
+      <c r="M48" s="11" t="inlineStr"/>
+      <c r="N48" s="11" t="inlineStr"/>
+      <c r="O48" s="11" t="inlineStr"/>
+      <c r="P48" s="12" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
@@ -1995,12 +2291,18 @@
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr"/>
-      <c r="E49" s="12" t="inlineStr"/>
-      <c r="F49" s="12" t="inlineStr"/>
+      <c r="E49" s="11" t="inlineStr"/>
+      <c r="F49" s="11" t="inlineStr"/>
       <c r="G49" s="11" t="inlineStr"/>
       <c r="H49" s="11" t="inlineStr"/>
-      <c r="I49" s="11" t="inlineStr"/>
+      <c r="I49" s="12" t="inlineStr"/>
       <c r="J49" s="12" t="inlineStr"/>
+      <c r="K49" s="11" t="inlineStr"/>
+      <c r="L49" s="11" t="inlineStr"/>
+      <c r="M49" s="11" t="inlineStr"/>
+      <c r="N49" s="11" t="inlineStr"/>
+      <c r="O49" s="11" t="inlineStr"/>
+      <c r="P49" s="12" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
@@ -2017,12 +2319,18 @@
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr"/>
-      <c r="E50" s="12" t="inlineStr"/>
-      <c r="F50" s="12" t="inlineStr"/>
+      <c r="E50" s="11" t="inlineStr"/>
+      <c r="F50" s="11" t="inlineStr"/>
       <c r="G50" s="11" t="inlineStr"/>
       <c r="H50" s="11" t="inlineStr"/>
-      <c r="I50" s="11" t="inlineStr"/>
+      <c r="I50" s="12" t="inlineStr"/>
       <c r="J50" s="12" t="inlineStr"/>
+      <c r="K50" s="11" t="inlineStr"/>
+      <c r="L50" s="11" t="inlineStr"/>
+      <c r="M50" s="11" t="inlineStr"/>
+      <c r="N50" s="11" t="inlineStr"/>
+      <c r="O50" s="11" t="inlineStr"/>
+      <c r="P50" s="12" t="inlineStr"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
@@ -2046,12 +2354,18 @@
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr"/>
-      <c r="E52" s="12" t="inlineStr"/>
-      <c r="F52" s="12" t="inlineStr"/>
+      <c r="E52" s="11" t="inlineStr"/>
+      <c r="F52" s="11" t="inlineStr"/>
       <c r="G52" s="11" t="inlineStr"/>
       <c r="H52" s="11" t="inlineStr"/>
-      <c r="I52" s="11" t="inlineStr"/>
+      <c r="I52" s="12" t="inlineStr"/>
       <c r="J52" s="12" t="inlineStr"/>
+      <c r="K52" s="11" t="inlineStr"/>
+      <c r="L52" s="11" t="inlineStr"/>
+      <c r="M52" s="11" t="inlineStr"/>
+      <c r="N52" s="11" t="inlineStr"/>
+      <c r="O52" s="11" t="inlineStr"/>
+      <c r="P52" s="12" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
@@ -2068,12 +2382,18 @@
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr"/>
-      <c r="E53" s="12" t="inlineStr"/>
-      <c r="F53" s="12" t="inlineStr"/>
+      <c r="E53" s="11" t="inlineStr"/>
+      <c r="F53" s="11" t="inlineStr"/>
       <c r="G53" s="11" t="inlineStr"/>
       <c r="H53" s="11" t="inlineStr"/>
-      <c r="I53" s="11" t="inlineStr"/>
+      <c r="I53" s="12" t="inlineStr"/>
       <c r="J53" s="12" t="inlineStr"/>
+      <c r="K53" s="11" t="inlineStr"/>
+      <c r="L53" s="11" t="inlineStr"/>
+      <c r="M53" s="11" t="inlineStr"/>
+      <c r="N53" s="11" t="inlineStr"/>
+      <c r="O53" s="11" t="inlineStr"/>
+      <c r="P53" s="12" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n">
@@ -2090,12 +2410,18 @@
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr"/>
-      <c r="E54" s="12" t="inlineStr"/>
-      <c r="F54" s="12" t="inlineStr"/>
+      <c r="E54" s="11" t="inlineStr"/>
+      <c r="F54" s="11" t="inlineStr"/>
       <c r="G54" s="11" t="inlineStr"/>
       <c r="H54" s="11" t="inlineStr"/>
-      <c r="I54" s="11" t="inlineStr"/>
+      <c r="I54" s="12" t="inlineStr"/>
       <c r="J54" s="12" t="inlineStr"/>
+      <c r="K54" s="11" t="inlineStr"/>
+      <c r="L54" s="11" t="inlineStr"/>
+      <c r="M54" s="11" t="inlineStr"/>
+      <c r="N54" s="11" t="inlineStr"/>
+      <c r="O54" s="11" t="inlineStr"/>
+      <c r="P54" s="12" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
@@ -2112,12 +2438,18 @@
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr"/>
-      <c r="E55" s="12" t="inlineStr"/>
-      <c r="F55" s="12" t="inlineStr"/>
+      <c r="E55" s="11" t="inlineStr"/>
+      <c r="F55" s="11" t="inlineStr"/>
       <c r="G55" s="11" t="inlineStr"/>
       <c r="H55" s="11" t="inlineStr"/>
-      <c r="I55" s="11" t="inlineStr"/>
+      <c r="I55" s="12" t="inlineStr"/>
       <c r="J55" s="12" t="inlineStr"/>
+      <c r="K55" s="11" t="inlineStr"/>
+      <c r="L55" s="11" t="inlineStr"/>
+      <c r="M55" s="11" t="inlineStr"/>
+      <c r="N55" s="11" t="inlineStr"/>
+      <c r="O55" s="11" t="inlineStr"/>
+      <c r="P55" s="12" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
@@ -2134,12 +2466,18 @@
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr"/>
-      <c r="E56" s="12" t="inlineStr"/>
-      <c r="F56" s="12" t="inlineStr"/>
+      <c r="E56" s="11" t="inlineStr"/>
+      <c r="F56" s="11" t="inlineStr"/>
       <c r="G56" s="11" t="inlineStr"/>
       <c r="H56" s="11" t="inlineStr"/>
-      <c r="I56" s="11" t="inlineStr"/>
+      <c r="I56" s="12" t="inlineStr"/>
       <c r="J56" s="12" t="inlineStr"/>
+      <c r="K56" s="11" t="inlineStr"/>
+      <c r="L56" s="11" t="inlineStr"/>
+      <c r="M56" s="11" t="inlineStr"/>
+      <c r="N56" s="11" t="inlineStr"/>
+      <c r="O56" s="11" t="inlineStr"/>
+      <c r="P56" s="12" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
@@ -2156,12 +2494,18 @@
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr"/>
-      <c r="E57" s="12" t="inlineStr"/>
-      <c r="F57" s="12" t="inlineStr"/>
+      <c r="E57" s="11" t="inlineStr"/>
+      <c r="F57" s="11" t="inlineStr"/>
       <c r="G57" s="11" t="inlineStr"/>
       <c r="H57" s="11" t="inlineStr"/>
-      <c r="I57" s="11" t="inlineStr"/>
+      <c r="I57" s="12" t="inlineStr"/>
       <c r="J57" s="12" t="inlineStr"/>
+      <c r="K57" s="11" t="inlineStr"/>
+      <c r="L57" s="11" t="inlineStr"/>
+      <c r="M57" s="11" t="inlineStr"/>
+      <c r="N57" s="11" t="inlineStr"/>
+      <c r="O57" s="11" t="inlineStr"/>
+      <c r="P57" s="12" t="inlineStr"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="8" t="inlineStr">
@@ -2185,12 +2529,18 @@
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr"/>
-      <c r="E59" s="12" t="inlineStr"/>
-      <c r="F59" s="12" t="inlineStr"/>
+      <c r="E59" s="11" t="inlineStr"/>
+      <c r="F59" s="11" t="inlineStr"/>
       <c r="G59" s="11" t="inlineStr"/>
       <c r="H59" s="11" t="inlineStr"/>
-      <c r="I59" s="11" t="inlineStr"/>
+      <c r="I59" s="12" t="inlineStr"/>
       <c r="J59" s="12" t="inlineStr"/>
+      <c r="K59" s="11" t="inlineStr"/>
+      <c r="L59" s="11" t="inlineStr"/>
+      <c r="M59" s="11" t="inlineStr"/>
+      <c r="N59" s="11" t="inlineStr"/>
+      <c r="O59" s="11" t="inlineStr"/>
+      <c r="P59" s="12" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n">
@@ -2207,12 +2557,18 @@
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr"/>
-      <c r="E60" s="12" t="inlineStr"/>
-      <c r="F60" s="12" t="inlineStr"/>
+      <c r="E60" s="11" t="inlineStr"/>
+      <c r="F60" s="11" t="inlineStr"/>
       <c r="G60" s="11" t="inlineStr"/>
       <c r="H60" s="11" t="inlineStr"/>
-      <c r="I60" s="11" t="inlineStr"/>
+      <c r="I60" s="12" t="inlineStr"/>
       <c r="J60" s="12" t="inlineStr"/>
+      <c r="K60" s="11" t="inlineStr"/>
+      <c r="L60" s="11" t="inlineStr"/>
+      <c r="M60" s="11" t="inlineStr"/>
+      <c r="N60" s="11" t="inlineStr"/>
+      <c r="O60" s="11" t="inlineStr"/>
+      <c r="P60" s="12" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
@@ -2229,12 +2585,18 @@
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr"/>
-      <c r="E61" s="12" t="inlineStr"/>
-      <c r="F61" s="12" t="inlineStr"/>
+      <c r="E61" s="11" t="inlineStr"/>
+      <c r="F61" s="11" t="inlineStr"/>
       <c r="G61" s="11" t="inlineStr"/>
       <c r="H61" s="11" t="inlineStr"/>
-      <c r="I61" s="11" t="inlineStr"/>
+      <c r="I61" s="12" t="inlineStr"/>
       <c r="J61" s="12" t="inlineStr"/>
+      <c r="K61" s="11" t="inlineStr"/>
+      <c r="L61" s="11" t="inlineStr"/>
+      <c r="M61" s="11" t="inlineStr"/>
+      <c r="N61" s="11" t="inlineStr"/>
+      <c r="O61" s="11" t="inlineStr"/>
+      <c r="P61" s="12" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n">
@@ -2251,12 +2613,18 @@
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr"/>
-      <c r="E62" s="12" t="inlineStr"/>
-      <c r="F62" s="12" t="inlineStr"/>
+      <c r="E62" s="11" t="inlineStr"/>
+      <c r="F62" s="11" t="inlineStr"/>
       <c r="G62" s="11" t="inlineStr"/>
       <c r="H62" s="11" t="inlineStr"/>
-      <c r="I62" s="11" t="inlineStr"/>
+      <c r="I62" s="12" t="inlineStr"/>
       <c r="J62" s="12" t="inlineStr"/>
+      <c r="K62" s="11" t="inlineStr"/>
+      <c r="L62" s="11" t="inlineStr"/>
+      <c r="M62" s="11" t="inlineStr"/>
+      <c r="N62" s="11" t="inlineStr"/>
+      <c r="O62" s="11" t="inlineStr"/>
+      <c r="P62" s="12" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
@@ -2273,12 +2641,18 @@
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr"/>
-      <c r="E63" s="12" t="inlineStr"/>
-      <c r="F63" s="12" t="inlineStr"/>
+      <c r="E63" s="11" t="inlineStr"/>
+      <c r="F63" s="11" t="inlineStr"/>
       <c r="G63" s="11" t="inlineStr"/>
       <c r="H63" s="11" t="inlineStr"/>
-      <c r="I63" s="11" t="inlineStr"/>
+      <c r="I63" s="12" t="inlineStr"/>
       <c r="J63" s="12" t="inlineStr"/>
+      <c r="K63" s="11" t="inlineStr"/>
+      <c r="L63" s="11" t="inlineStr"/>
+      <c r="M63" s="11" t="inlineStr"/>
+      <c r="N63" s="11" t="inlineStr"/>
+      <c r="O63" s="11" t="inlineStr"/>
+      <c r="P63" s="12" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
@@ -2295,12 +2669,18 @@
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr"/>
-      <c r="E64" s="12" t="inlineStr"/>
-      <c r="F64" s="12" t="inlineStr"/>
+      <c r="E64" s="11" t="inlineStr"/>
+      <c r="F64" s="11" t="inlineStr"/>
       <c r="G64" s="11" t="inlineStr"/>
       <c r="H64" s="11" t="inlineStr"/>
-      <c r="I64" s="11" t="inlineStr"/>
+      <c r="I64" s="12" t="inlineStr"/>
       <c r="J64" s="12" t="inlineStr"/>
+      <c r="K64" s="11" t="inlineStr"/>
+      <c r="L64" s="11" t="inlineStr"/>
+      <c r="M64" s="11" t="inlineStr"/>
+      <c r="N64" s="11" t="inlineStr"/>
+      <c r="O64" s="11" t="inlineStr"/>
+      <c r="P64" s="12" t="inlineStr"/>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="8" t="inlineStr">
@@ -2324,12 +2704,18 @@
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr"/>
-      <c r="E66" s="12" t="inlineStr"/>
-      <c r="F66" s="12" t="inlineStr"/>
+      <c r="E66" s="11" t="inlineStr"/>
+      <c r="F66" s="11" t="inlineStr"/>
       <c r="G66" s="11" t="inlineStr"/>
       <c r="H66" s="11" t="inlineStr"/>
-      <c r="I66" s="11" t="inlineStr"/>
+      <c r="I66" s="12" t="inlineStr"/>
       <c r="J66" s="12" t="inlineStr"/>
+      <c r="K66" s="11" t="inlineStr"/>
+      <c r="L66" s="11" t="inlineStr"/>
+      <c r="M66" s="11" t="inlineStr"/>
+      <c r="N66" s="11" t="inlineStr"/>
+      <c r="O66" s="11" t="inlineStr"/>
+      <c r="P66" s="12" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
@@ -2346,12 +2732,18 @@
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr"/>
-      <c r="E67" s="12" t="inlineStr"/>
-      <c r="F67" s="12" t="inlineStr"/>
+      <c r="E67" s="11" t="inlineStr"/>
+      <c r="F67" s="11" t="inlineStr"/>
       <c r="G67" s="11" t="inlineStr"/>
       <c r="H67" s="11" t="inlineStr"/>
-      <c r="I67" s="11" t="inlineStr"/>
+      <c r="I67" s="12" t="inlineStr"/>
       <c r="J67" s="12" t="inlineStr"/>
+      <c r="K67" s="11" t="inlineStr"/>
+      <c r="L67" s="11" t="inlineStr"/>
+      <c r="M67" s="11" t="inlineStr"/>
+      <c r="N67" s="11" t="inlineStr"/>
+      <c r="O67" s="11" t="inlineStr"/>
+      <c r="P67" s="12" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
@@ -2368,12 +2760,18 @@
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr"/>
-      <c r="E68" s="12" t="inlineStr"/>
-      <c r="F68" s="12" t="inlineStr"/>
+      <c r="E68" s="11" t="inlineStr"/>
+      <c r="F68" s="11" t="inlineStr"/>
       <c r="G68" s="11" t="inlineStr"/>
       <c r="H68" s="11" t="inlineStr"/>
-      <c r="I68" s="11" t="inlineStr"/>
+      <c r="I68" s="12" t="inlineStr"/>
       <c r="J68" s="12" t="inlineStr"/>
+      <c r="K68" s="11" t="inlineStr"/>
+      <c r="L68" s="11" t="inlineStr"/>
+      <c r="M68" s="11" t="inlineStr"/>
+      <c r="N68" s="11" t="inlineStr"/>
+      <c r="O68" s="11" t="inlineStr"/>
+      <c r="P68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n">
@@ -2390,12 +2788,18 @@
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr"/>
-      <c r="E69" s="12" t="inlineStr"/>
-      <c r="F69" s="12" t="inlineStr"/>
+      <c r="E69" s="11" t="inlineStr"/>
+      <c r="F69" s="11" t="inlineStr"/>
       <c r="G69" s="11" t="inlineStr"/>
       <c r="H69" s="11" t="inlineStr"/>
-      <c r="I69" s="11" t="inlineStr"/>
+      <c r="I69" s="12" t="inlineStr"/>
       <c r="J69" s="12" t="inlineStr"/>
+      <c r="K69" s="11" t="inlineStr"/>
+      <c r="L69" s="11" t="inlineStr"/>
+      <c r="M69" s="11" t="inlineStr"/>
+      <c r="N69" s="11" t="inlineStr"/>
+      <c r="O69" s="11" t="inlineStr"/>
+      <c r="P69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n">
@@ -2412,12 +2816,18 @@
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr"/>
-      <c r="E70" s="12" t="inlineStr"/>
-      <c r="F70" s="12" t="inlineStr"/>
+      <c r="E70" s="11" t="inlineStr"/>
+      <c r="F70" s="11" t="inlineStr"/>
       <c r="G70" s="11" t="inlineStr"/>
       <c r="H70" s="11" t="inlineStr"/>
-      <c r="I70" s="11" t="inlineStr"/>
+      <c r="I70" s="12" t="inlineStr"/>
       <c r="J70" s="12" t="inlineStr"/>
+      <c r="K70" s="11" t="inlineStr"/>
+      <c r="L70" s="11" t="inlineStr"/>
+      <c r="M70" s="11" t="inlineStr"/>
+      <c r="N70" s="11" t="inlineStr"/>
+      <c r="O70" s="11" t="inlineStr"/>
+      <c r="P70" s="12" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
@@ -2434,12 +2844,18 @@
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
-      <c r="E71" s="12" t="inlineStr"/>
-      <c r="F71" s="12" t="inlineStr"/>
+      <c r="E71" s="11" t="inlineStr"/>
+      <c r="F71" s="11" t="inlineStr"/>
       <c r="G71" s="11" t="inlineStr"/>
       <c r="H71" s="11" t="inlineStr"/>
-      <c r="I71" s="11" t="inlineStr"/>
+      <c r="I71" s="12" t="inlineStr"/>
       <c r="J71" s="12" t="inlineStr"/>
+      <c r="K71" s="11" t="inlineStr"/>
+      <c r="L71" s="11" t="inlineStr"/>
+      <c r="M71" s="11" t="inlineStr"/>
+      <c r="N71" s="11" t="inlineStr"/>
+      <c r="O71" s="11" t="inlineStr"/>
+      <c r="P71" s="12" t="inlineStr"/>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="8" t="inlineStr">
@@ -2463,12 +2879,18 @@
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
-      <c r="E73" s="12" t="inlineStr"/>
-      <c r="F73" s="12" t="inlineStr"/>
+      <c r="E73" s="11" t="inlineStr"/>
+      <c r="F73" s="11" t="inlineStr"/>
       <c r="G73" s="11" t="inlineStr"/>
       <c r="H73" s="11" t="inlineStr"/>
-      <c r="I73" s="11" t="inlineStr"/>
+      <c r="I73" s="12" t="inlineStr"/>
       <c r="J73" s="12" t="inlineStr"/>
+      <c r="K73" s="11" t="inlineStr"/>
+      <c r="L73" s="11" t="inlineStr"/>
+      <c r="M73" s="11" t="inlineStr"/>
+      <c r="N73" s="11" t="inlineStr"/>
+      <c r="O73" s="11" t="inlineStr"/>
+      <c r="P73" s="12" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n">
@@ -2485,12 +2907,18 @@
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
-      <c r="E74" s="12" t="inlineStr"/>
-      <c r="F74" s="12" t="inlineStr"/>
+      <c r="E74" s="11" t="inlineStr"/>
+      <c r="F74" s="11" t="inlineStr"/>
       <c r="G74" s="11" t="inlineStr"/>
       <c r="H74" s="11" t="inlineStr"/>
-      <c r="I74" s="11" t="inlineStr"/>
+      <c r="I74" s="12" t="inlineStr"/>
       <c r="J74" s="12" t="inlineStr"/>
+      <c r="K74" s="11" t="inlineStr"/>
+      <c r="L74" s="11" t="inlineStr"/>
+      <c r="M74" s="11" t="inlineStr"/>
+      <c r="N74" s="11" t="inlineStr"/>
+      <c r="O74" s="11" t="inlineStr"/>
+      <c r="P74" s="12" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
@@ -2507,12 +2935,18 @@
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
-      <c r="E75" s="12" t="inlineStr"/>
-      <c r="F75" s="12" t="inlineStr"/>
+      <c r="E75" s="11" t="inlineStr"/>
+      <c r="F75" s="11" t="inlineStr"/>
       <c r="G75" s="11" t="inlineStr"/>
       <c r="H75" s="11" t="inlineStr"/>
-      <c r="I75" s="11" t="inlineStr"/>
+      <c r="I75" s="12" t="inlineStr"/>
       <c r="J75" s="12" t="inlineStr"/>
+      <c r="K75" s="11" t="inlineStr"/>
+      <c r="L75" s="11" t="inlineStr"/>
+      <c r="M75" s="11" t="inlineStr"/>
+      <c r="N75" s="11" t="inlineStr"/>
+      <c r="O75" s="11" t="inlineStr"/>
+      <c r="P75" s="12" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="9" t="n">
@@ -2529,12 +2963,18 @@
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
-      <c r="E76" s="12" t="inlineStr"/>
-      <c r="F76" s="12" t="inlineStr"/>
+      <c r="E76" s="11" t="inlineStr"/>
+      <c r="F76" s="11" t="inlineStr"/>
       <c r="G76" s="11" t="inlineStr"/>
       <c r="H76" s="11" t="inlineStr"/>
-      <c r="I76" s="11" t="inlineStr"/>
+      <c r="I76" s="12" t="inlineStr"/>
       <c r="J76" s="12" t="inlineStr"/>
+      <c r="K76" s="11" t="inlineStr"/>
+      <c r="L76" s="11" t="inlineStr"/>
+      <c r="M76" s="11" t="inlineStr"/>
+      <c r="N76" s="11" t="inlineStr"/>
+      <c r="O76" s="11" t="inlineStr"/>
+      <c r="P76" s="12" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
@@ -2551,12 +2991,18 @@
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
-      <c r="E77" s="12" t="inlineStr"/>
-      <c r="F77" s="12" t="inlineStr"/>
+      <c r="E77" s="11" t="inlineStr"/>
+      <c r="F77" s="11" t="inlineStr"/>
       <c r="G77" s="11" t="inlineStr"/>
       <c r="H77" s="11" t="inlineStr"/>
-      <c r="I77" s="11" t="inlineStr"/>
+      <c r="I77" s="12" t="inlineStr"/>
       <c r="J77" s="12" t="inlineStr"/>
+      <c r="K77" s="11" t="inlineStr"/>
+      <c r="L77" s="11" t="inlineStr"/>
+      <c r="M77" s="11" t="inlineStr"/>
+      <c r="N77" s="11" t="inlineStr"/>
+      <c r="O77" s="11" t="inlineStr"/>
+      <c r="P77" s="12" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="9" t="n">
@@ -2573,12 +3019,18 @@
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr"/>
-      <c r="E78" s="12" t="inlineStr"/>
-      <c r="F78" s="12" t="inlineStr"/>
+      <c r="E78" s="11" t="inlineStr"/>
+      <c r="F78" s="11" t="inlineStr"/>
       <c r="G78" s="11" t="inlineStr"/>
       <c r="H78" s="11" t="inlineStr"/>
-      <c r="I78" s="11" t="inlineStr"/>
+      <c r="I78" s="12" t="inlineStr"/>
       <c r="J78" s="12" t="inlineStr"/>
+      <c r="K78" s="11" t="inlineStr"/>
+      <c r="L78" s="11" t="inlineStr"/>
+      <c r="M78" s="11" t="inlineStr"/>
+      <c r="N78" s="11" t="inlineStr"/>
+      <c r="O78" s="11" t="inlineStr"/>
+      <c r="P78" s="12" t="inlineStr"/>
     </row>
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="8" t="inlineStr">
@@ -2602,12 +3054,18 @@
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr"/>
-      <c r="E80" s="12" t="inlineStr"/>
-      <c r="F80" s="12" t="inlineStr"/>
+      <c r="E80" s="11" t="inlineStr"/>
+      <c r="F80" s="11" t="inlineStr"/>
       <c r="G80" s="11" t="inlineStr"/>
       <c r="H80" s="11" t="inlineStr"/>
-      <c r="I80" s="11" t="inlineStr"/>
+      <c r="I80" s="12" t="inlineStr"/>
       <c r="J80" s="12" t="inlineStr"/>
+      <c r="K80" s="11" t="inlineStr"/>
+      <c r="L80" s="11" t="inlineStr"/>
+      <c r="M80" s="11" t="inlineStr"/>
+      <c r="N80" s="11" t="inlineStr"/>
+      <c r="O80" s="11" t="inlineStr"/>
+      <c r="P80" s="12" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
@@ -2624,12 +3082,18 @@
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr"/>
-      <c r="E81" s="12" t="inlineStr"/>
-      <c r="F81" s="12" t="inlineStr"/>
+      <c r="E81" s="11" t="inlineStr"/>
+      <c r="F81" s="11" t="inlineStr"/>
       <c r="G81" s="11" t="inlineStr"/>
       <c r="H81" s="11" t="inlineStr"/>
-      <c r="I81" s="11" t="inlineStr"/>
+      <c r="I81" s="12" t="inlineStr"/>
       <c r="J81" s="12" t="inlineStr"/>
+      <c r="K81" s="11" t="inlineStr"/>
+      <c r="L81" s="11" t="inlineStr"/>
+      <c r="M81" s="11" t="inlineStr"/>
+      <c r="N81" s="11" t="inlineStr"/>
+      <c r="O81" s="11" t="inlineStr"/>
+      <c r="P81" s="12" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n">
@@ -2646,12 +3110,18 @@
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr"/>
-      <c r="E82" s="12" t="inlineStr"/>
-      <c r="F82" s="12" t="inlineStr"/>
+      <c r="E82" s="11" t="inlineStr"/>
+      <c r="F82" s="11" t="inlineStr"/>
       <c r="G82" s="11" t="inlineStr"/>
       <c r="H82" s="11" t="inlineStr"/>
-      <c r="I82" s="11" t="inlineStr"/>
+      <c r="I82" s="12" t="inlineStr"/>
       <c r="J82" s="12" t="inlineStr"/>
+      <c r="K82" s="11" t="inlineStr"/>
+      <c r="L82" s="11" t="inlineStr"/>
+      <c r="M82" s="11" t="inlineStr"/>
+      <c r="N82" s="11" t="inlineStr"/>
+      <c r="O82" s="11" t="inlineStr"/>
+      <c r="P82" s="12" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n">
@@ -2668,12 +3138,18 @@
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr"/>
-      <c r="E83" s="12" t="inlineStr"/>
-      <c r="F83" s="12" t="inlineStr"/>
+      <c r="E83" s="11" t="inlineStr"/>
+      <c r="F83" s="11" t="inlineStr"/>
       <c r="G83" s="11" t="inlineStr"/>
       <c r="H83" s="11" t="inlineStr"/>
-      <c r="I83" s="11" t="inlineStr"/>
+      <c r="I83" s="12" t="inlineStr"/>
       <c r="J83" s="12" t="inlineStr"/>
+      <c r="K83" s="11" t="inlineStr"/>
+      <c r="L83" s="11" t="inlineStr"/>
+      <c r="M83" s="11" t="inlineStr"/>
+      <c r="N83" s="11" t="inlineStr"/>
+      <c r="O83" s="11" t="inlineStr"/>
+      <c r="P83" s="12" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="9" t="n">
@@ -2690,12 +3166,18 @@
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr"/>
-      <c r="E84" s="12" t="inlineStr"/>
-      <c r="F84" s="12" t="inlineStr"/>
+      <c r="E84" s="11" t="inlineStr"/>
+      <c r="F84" s="11" t="inlineStr"/>
       <c r="G84" s="11" t="inlineStr"/>
       <c r="H84" s="11" t="inlineStr"/>
-      <c r="I84" s="11" t="inlineStr"/>
+      <c r="I84" s="12" t="inlineStr"/>
       <c r="J84" s="12" t="inlineStr"/>
+      <c r="K84" s="11" t="inlineStr"/>
+      <c r="L84" s="11" t="inlineStr"/>
+      <c r="M84" s="11" t="inlineStr"/>
+      <c r="N84" s="11" t="inlineStr"/>
+      <c r="O84" s="11" t="inlineStr"/>
+      <c r="P84" s="12" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
@@ -2712,29 +3194,35 @@
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr"/>
-      <c r="E85" s="12" t="inlineStr"/>
-      <c r="F85" s="12" t="inlineStr"/>
+      <c r="E85" s="11" t="inlineStr"/>
+      <c r="F85" s="11" t="inlineStr"/>
       <c r="G85" s="11" t="inlineStr"/>
       <c r="H85" s="11" t="inlineStr"/>
-      <c r="I85" s="11" t="inlineStr"/>
+      <c r="I85" s="12" t="inlineStr"/>
       <c r="J85" s="12" t="inlineStr"/>
+      <c r="K85" s="11" t="inlineStr"/>
+      <c r="L85" s="11" t="inlineStr"/>
+      <c r="M85" s="11" t="inlineStr"/>
+      <c r="N85" s="11" t="inlineStr"/>
+      <c r="O85" s="11" t="inlineStr"/>
+      <c r="P85" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A44:J44"/>
-    <mergeCell ref="A23:J23"/>
-    <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A79:J79"/>
-    <mergeCell ref="A58:J58"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A30:J30"/>
-    <mergeCell ref="A65:J65"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="A72:J72"/>
-    <mergeCell ref="A51:J51"/>
+    <mergeCell ref="A51:P51"/>
+    <mergeCell ref="A44:P44"/>
+    <mergeCell ref="A23:P23"/>
+    <mergeCell ref="A9:P9"/>
+    <mergeCell ref="A37:P37"/>
+    <mergeCell ref="A79:P79"/>
+    <mergeCell ref="A58:P58"/>
+    <mergeCell ref="A30:P30"/>
+    <mergeCell ref="A16:P16"/>
+    <mergeCell ref="A72:P72"/>
+    <mergeCell ref="A65:P65"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I2:I85">
+  <conditionalFormatting sqref="O2:O85">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"At risk"</formula>
     </cfRule>
@@ -2745,14 +3233,32 @@
       <formula>"On track"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations count="9">
     <dataValidation sqref="D2:D85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No,Excused"</formula1>
+      <formula1>"0,1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0,1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0,1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0,1,2,3,4,5"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0,1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"0,1,2,3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0,1,2,3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"On track,Watch,At risk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3027,7 +3533,7 @@
         </is>
       </c>
       <c r="Y2" s="13">
-        <f>IF(B2="","",SUMIF('Weekly Tracker'!$C:$C,B2,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B2="","",SUMIF('Weekly Tracker'!$C:$C,B2,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3135,7 +3641,7 @@
         </is>
       </c>
       <c r="Y3" s="13">
-        <f>IF(B3="","",SUMIF('Weekly Tracker'!$C:$C,B3,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B3="","",SUMIF('Weekly Tracker'!$C:$C,B3,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3243,7 +3749,7 @@
         </is>
       </c>
       <c r="Y4" s="13">
-        <f>IF(B4="","",SUMIF('Weekly Tracker'!$C:$C,B4,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B4="","",SUMIF('Weekly Tracker'!$C:$C,B4,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3351,7 +3857,7 @@
         </is>
       </c>
       <c r="Y5" s="13">
-        <f>IF(B5="","",SUMIF('Weekly Tracker'!$C:$C,B5,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B5="","",SUMIF('Weekly Tracker'!$C:$C,B5,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3459,7 +3965,7 @@
         </is>
       </c>
       <c r="Y6" s="13">
-        <f>IF(B6="","",SUMIF('Weekly Tracker'!$C:$C,B6,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B6="","",SUMIF('Weekly Tracker'!$C:$C,B6,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3567,7 +4073,7 @@
         </is>
       </c>
       <c r="Y7" s="13">
-        <f>IF(B7="","",SUMIF('Weekly Tracker'!$C:$C,B7,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B7="","",SUMIF('Weekly Tracker'!$C:$C,B7,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3597,7 +4103,7 @@
       <c r="W8" s="11" t="inlineStr"/>
       <c r="X8" s="12" t="inlineStr"/>
       <c r="Y8" s="13">
-        <f>IF(B8="","",SUMIF('Weekly Tracker'!$C:$C,B8,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B8="","",SUMIF('Weekly Tracker'!$C:$C,B8,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3627,7 +4133,7 @@
       <c r="W9" s="11" t="inlineStr"/>
       <c r="X9" s="12" t="inlineStr"/>
       <c r="Y9" s="13">
-        <f>IF(B9="","",SUMIF('Weekly Tracker'!$C:$C,B9,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B9="","",SUMIF('Weekly Tracker'!$C:$C,B9,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3657,7 +4163,7 @@
       <c r="W10" s="11" t="inlineStr"/>
       <c r="X10" s="12" t="inlineStr"/>
       <c r="Y10" s="13">
-        <f>IF(B10="","",SUMIF('Weekly Tracker'!$C:$C,B10,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B10="","",SUMIF('Weekly Tracker'!$C:$C,B10,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3687,7 +4193,7 @@
       <c r="W11" s="11" t="inlineStr"/>
       <c r="X11" s="12" t="inlineStr"/>
       <c r="Y11" s="13">
-        <f>IF(B11="","",SUMIF('Weekly Tracker'!$C:$C,B11,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B11="","",SUMIF('Weekly Tracker'!$C:$C,B11,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3717,7 +4223,7 @@
       <c r="W12" s="11" t="inlineStr"/>
       <c r="X12" s="12" t="inlineStr"/>
       <c r="Y12" s="13">
-        <f>IF(B12="","",SUMIF('Weekly Tracker'!$C:$C,B12,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B12="","",SUMIF('Weekly Tracker'!$C:$C,B12,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3747,7 +4253,7 @@
       <c r="W13" s="11" t="inlineStr"/>
       <c r="X13" s="12" t="inlineStr"/>
       <c r="Y13" s="13">
-        <f>IF(B13="","",SUMIF('Weekly Tracker'!$C:$C,B13,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B13="","",SUMIF('Weekly Tracker'!$C:$C,B13,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3777,7 +4283,7 @@
       <c r="W14" s="11" t="inlineStr"/>
       <c r="X14" s="12" t="inlineStr"/>
       <c r="Y14" s="13">
-        <f>IF(B14="","",SUMIF('Weekly Tracker'!$C:$C,B14,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B14="","",SUMIF('Weekly Tracker'!$C:$C,B14,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3807,7 +4313,7 @@
       <c r="W15" s="11" t="inlineStr"/>
       <c r="X15" s="12" t="inlineStr"/>
       <c r="Y15" s="13">
-        <f>IF(B15="","",SUMIF('Weekly Tracker'!$C:$C,B15,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B15="","",SUMIF('Weekly Tracker'!$C:$C,B15,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3837,7 +4343,7 @@
       <c r="W16" s="11" t="inlineStr"/>
       <c r="X16" s="12" t="inlineStr"/>
       <c r="Y16" s="13">
-        <f>IF(B16="","",SUMIF('Weekly Tracker'!$C:$C,B16,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B16="","",SUMIF('Weekly Tracker'!$C:$C,B16,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3867,7 +4373,7 @@
       <c r="W17" s="11" t="inlineStr"/>
       <c r="X17" s="12" t="inlineStr"/>
       <c r="Y17" s="13">
-        <f>IF(B17="","",SUMIF('Weekly Tracker'!$C:$C,B17,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B17="","",SUMIF('Weekly Tracker'!$C:$C,B17,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3897,7 +4403,7 @@
       <c r="W18" s="11" t="inlineStr"/>
       <c r="X18" s="12" t="inlineStr"/>
       <c r="Y18" s="13">
-        <f>IF(B18="","",SUMIF('Weekly Tracker'!$C:$C,B18,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B18="","",SUMIF('Weekly Tracker'!$C:$C,B18,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>
@@ -3927,7 +4433,7 @@
       <c r="W19" s="11" t="inlineStr"/>
       <c r="X19" s="12" t="inlineStr"/>
       <c r="Y19" s="13">
-        <f>IF(B19="","",SUMIF('Weekly Tracker'!$C:$C,B19,'Weekly Tracker'!$H:$H))</f>
+        <f>IF(B19="","",SUMIF('Weekly Tracker'!$C:$C,B19,'Weekly Tracker'!$N:$N))</f>
         <v/>
       </c>
     </row>

</xml_diff>